<commit_message>
Refresh schedule analyzer sample files
</commit_message>
<xml_diff>
--- a/assets/data/sample-smartsheet-schedule-input.xlsx
+++ b/assets/data/sample-smartsheet-schedule-input.xlsx
@@ -1,6 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr/>
   <sheets>
     <sheet name="Sample Schedule Export" sheetId="1" r:id="rId1"/>
   </sheets>
@@ -9,15 +10,27 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="1">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
@@ -32,9 +45,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -44,7 +58,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -54,57 +68,68 @@
     <col min="5" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="2">
         <is>
           <t>Project Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="2">
         <is>
           <t>Task ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="2">
         <is>
           <t>Task Name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="2">
         <is>
           <t>Hierarchy Level</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="2">
         <is>
           <t>Baseline Start</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="2">
         <is>
           <t>Baseline Finish</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="2">
         <is>
           <t>Current Start</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" t="inlineStr" s="2">
         <is>
           <t>Current Finish</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" t="inlineStr" s="2">
         <is>
           <t>Predecessors</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" t="inlineStr" s="2">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="2">
+        <is>
+          <t>Row Type</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="2">
+        <is>
+          <t>Include in Critical Path?</t>
         </is>
       </c>
     </row>
@@ -116,28 +141,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LOB-000</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sample Lobby Refresh Summary</t>
+          <t>Sample Lobby Refresh</t>
         </is>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" s="1">
-        <v>46028</v>
+        <v>46027</v>
       </c>
       <c r="F2" s="1">
+        <v>46050</v>
+      </c>
+      <c r="G2" s="1">
+        <v>46027</v>
+      </c>
+      <c r="H2" s="1">
         <v>46051</v>
-      </c>
-      <c r="G2" s="1">
-        <v>46028</v>
-      </c>
-      <c r="H2" s="1">
-        <v>46052</v>
       </c>
       <c r="I2"/>
       <c r="J2" t="inlineStr">
@@ -145,6 +170,12 @@
           <t>In Progress</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="L2"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -154,28 +185,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LOB-010</t>
+          <t>L-001</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Kickoff and site review</t>
+          <t>Project kickoff and site review</t>
         </is>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="E3" s="1">
-        <v>46028</v>
+        <v>46027</v>
       </c>
       <c r="F3" s="1">
-        <v>46028</v>
+        <v>46027</v>
       </c>
       <c r="G3" s="1">
-        <v>46028</v>
+        <v>46027</v>
       </c>
       <c r="H3" s="1">
-        <v>46028</v>
+        <v>46027</v>
       </c>
       <c r="I3"/>
       <c r="J3" t="inlineStr">
@@ -183,6 +214,12 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="L3"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -192,29 +229,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LOB-020</t>
+          <t>L-002</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Order finish materials</t>
+          <t>Order lobby finish materials</t>
         </is>
       </c>
       <c r="D4">
         <v>2</v>
       </c>
       <c r="E4" s="1">
-        <v>46029</v>
+        <v>46028</v>
       </c>
       <c r="F4" s="1">
+        <v>46030</v>
+      </c>
+      <c r="G4" s="1">
+        <v>46028</v>
+      </c>
+      <c r="H4" s="1">
         <v>46031</v>
       </c>
-      <c r="G4" s="1">
-        <v>46030</v>
-      </c>
-      <c r="H4" s="1">
-        <v>46035</v>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>2</t>
@@ -222,9 +259,15 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>In Progress</t>
-        </is>
-      </c>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="L4"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -234,7 +277,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LOB-030</t>
+          <t>L-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -246,16 +289,16 @@
         <v>2</v>
       </c>
       <c r="E5" s="1">
-        <v>46032</v>
+        <v>46031</v>
       </c>
       <c r="F5" s="1">
-        <v>46034</v>
+        <v>46031</v>
       </c>
       <c r="G5" s="1">
-        <v>46035</v>
+        <v>46031</v>
       </c>
       <c r="H5" s="1">
-        <v>46036</v>
+        <v>46031</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -264,9 +307,15 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>In Progress</t>
-        </is>
-      </c>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="L5"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -276,7 +325,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LOB-040</t>
+          <t>L-004</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -288,10 +337,10 @@
         <v>2</v>
       </c>
       <c r="E6" s="1">
-        <v>46035</v>
+        <v>46034</v>
       </c>
       <c r="F6" s="1">
-        <v>46039</v>
+        <v>46036</v>
       </c>
       <c r="G6" s="1">
         <v>46036</v>
@@ -306,9 +355,15 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>In Progress</t>
-        </is>
-      </c>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="L6"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -318,39 +373,45 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LOB-050</t>
+          <t>L-SPEND-01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wall prep and paint</t>
+          <t>Lobby budget check-in</t>
         </is>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" s="1">
-        <v>46040</v>
+        <v>46034</v>
       </c>
       <c r="F7" s="1">
-        <v>46044</v>
+        <v>46034</v>
       </c>
       <c r="G7" s="1">
-        <v>46039</v>
+        <v>46035</v>
       </c>
       <c r="H7" s="1">
-        <v>46044</v>
+        <v>46035</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>5SS</t>
+          <t>3FS</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="L7"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -360,35 +421,45 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LOB-060</t>
+          <t>L-005</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lighting refresh package</t>
+          <t>Wall prep and paint</t>
         </is>
       </c>
       <c r="D8">
         <v>2</v>
       </c>
       <c r="E8" s="1">
-        <v>46045</v>
+        <v>46037</v>
       </c>
       <c r="F8" s="1">
-        <v>46050</v>
+        <v>46042</v>
       </c>
       <c r="G8" s="1">
-        <v>46046</v>
+        <v>46036</v>
       </c>
       <c r="H8" s="1">
-        <v>46052</v>
-      </c>
-      <c r="I8"/>
+        <v>46042</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>5SS</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="L8"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -398,39 +469,45 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LOB-070</t>
+          <t>L-006</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Remove old fixtures</t>
+          <t>Lighting refresh milestone</t>
         </is>
       </c>
       <c r="D9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" s="1">
-        <v>46045</v>
+        <v>46043</v>
       </c>
       <c r="F9" s="1">
-        <v>46046</v>
+        <v>46043</v>
       </c>
       <c r="G9" s="1">
-        <v>46046</v>
+        <v>46042</v>
       </c>
       <c r="H9" s="1">
-        <v>46047</v>
+        <v>46042</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>6FS</t>
+          <t>3FS</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="L9"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -440,39 +517,45 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LOB-080</t>
+          <t>L-REPORT-01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Install new fixtures</t>
+          <t>Weekly lobby status update</t>
         </is>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" s="1">
-        <v>46047</v>
+        <v>46038</v>
       </c>
       <c r="F10" s="1">
-        <v>46049</v>
+        <v>46038</v>
       </c>
       <c r="G10" s="1">
-        <v>46046</v>
+        <v>46038</v>
       </c>
       <c r="H10" s="1">
-        <v>46048</v>
+        <v>46038</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>8FS</t>
+          <t>7FS</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+      <c r="L10"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -482,115 +565,141 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LOB-090</t>
+          <t>L-007</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Final walkthrough</t>
+          <t>Remove old light fixtures</t>
         </is>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
       <c r="E11" s="1">
-        <v>46050</v>
+        <v>46043</v>
       </c>
       <c r="F11" s="1">
-        <v>46051</v>
+        <v>46044</v>
       </c>
       <c r="G11" s="1">
-        <v>46051</v>
+        <v>46044</v>
       </c>
       <c r="H11" s="1">
-        <v>46052</v>
+        <v>46045</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>9FS</t>
+          <t>4FS</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="L11"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sample Pool Repairs</t>
+          <t>Sample Lobby Refresh</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>POOL-000</t>
+          <t>L-008</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Sample Pool Repairs Summary</t>
+          <t>Install new light fixtures</t>
         </is>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" s="1">
-        <v>46055</v>
+        <v>46045</v>
       </c>
       <c r="F12" s="1">
-        <v>46070</v>
+        <v>46049</v>
       </c>
       <c r="G12" s="1">
-        <v>46055</v>
+        <v>46048</v>
       </c>
       <c r="H12" s="1">
-        <v>46071</v>
-      </c>
-      <c r="I12"/>
+        <v>46050</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>10FS</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>In Progress</t>
-        </is>
-      </c>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="L12"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sample Pool Repairs</t>
+          <t>Sample Lobby Refresh</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>POOL-010</t>
+          <t>L-009</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Scope confirmation</t>
+          <t>Final lobby walkthrough milestone</t>
         </is>
       </c>
       <c r="D13">
         <v>2</v>
       </c>
       <c r="E13" s="1">
-        <v>46055</v>
+        <v>46050</v>
       </c>
       <c r="F13" s="1">
-        <v>46055</v>
+        <v>46050</v>
       </c>
       <c r="G13" s="1">
-        <v>46055</v>
+        <v>46051</v>
       </c>
       <c r="H13" s="1">
-        <v>46055</v>
-      </c>
-      <c r="I13"/>
+        <v>46051</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>8FS,11FS</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Complete</t>
-        </is>
-      </c>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="L13"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -600,39 +709,41 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>POOL-020</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Drain and clean pool</t>
+          <t>Sample Pool Repairs</t>
         </is>
       </c>
       <c r="D14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="1">
-        <v>46056</v>
+        <v>46055</v>
       </c>
       <c r="F14" s="1">
-        <v>46057</v>
+        <v>46076</v>
       </c>
       <c r="G14" s="1">
-        <v>46056</v>
+        <v>46055</v>
       </c>
       <c r="H14" s="1">
-        <v>46058</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
+        <v>46077</v>
+      </c>
+      <c r="I14"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="L14"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -642,39 +753,41 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>POOL-030</t>
+          <t>P-001</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Surface inspection</t>
+          <t>Confirm repair scope</t>
         </is>
       </c>
       <c r="D15">
         <v>2</v>
       </c>
       <c r="E15" s="1">
-        <v>46058</v>
+        <v>46055</v>
       </c>
       <c r="F15" s="1">
-        <v>46058</v>
+        <v>46055</v>
       </c>
       <c r="G15" s="1">
-        <v>46059</v>
+        <v>46055</v>
       </c>
       <c r="H15" s="1">
-        <v>46059</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>13FS</t>
-        </is>
-      </c>
+        <v>46055</v>
+      </c>
+      <c r="I15"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>In Progress</t>
-        </is>
-      </c>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="L15"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -684,39 +797,45 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>POOL-040</t>
+          <t>P-002</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Crack repair prep</t>
+          <t>Drain and clean pool</t>
         </is>
       </c>
       <c r="D16">
         <v>2</v>
       </c>
       <c r="E16" s="1">
-        <v>46059</v>
+        <v>46056</v>
       </c>
       <c r="F16" s="1">
-        <v>46061</v>
+        <v>46057</v>
       </c>
       <c r="G16" s="1">
-        <v>46060</v>
+        <v>46056</v>
       </c>
       <c r="H16" s="1">
-        <v>46061</v>
+        <v>46058</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>14FS+2d</t>
+          <t>14</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>In Progress</t>
-        </is>
-      </c>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="L16"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -726,35 +845,45 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>POOL-050</t>
+          <t>P-003</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tile repair package</t>
+          <t>Surface inspection</t>
         </is>
       </c>
       <c r="D17">
         <v>2</v>
       </c>
       <c r="E17" s="1">
-        <v>46062</v>
+        <v>46058</v>
       </c>
       <c r="F17" s="1">
-        <v>46067</v>
+        <v>46060</v>
       </c>
       <c r="G17" s="1">
-        <v>46061</v>
+        <v>46059</v>
       </c>
       <c r="H17" s="1">
-        <v>46067</v>
-      </c>
-      <c r="I17"/>
+        <v>46059</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>15FS</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="L17"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -764,16 +893,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>POOL-060</t>
+          <t>P-004</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Remove damaged tile</t>
+          <t>Crack repair prep</t>
         </is>
       </c>
       <c r="D18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E18" s="1">
         <v>46062</v>
@@ -782,21 +911,27 @@
         <v>46063</v>
       </c>
       <c r="G18" s="1">
-        <v>46061</v>
+        <v>46062</v>
       </c>
       <c r="H18" s="1">
         <v>46062</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>15SS</t>
+          <t>16FS+2d</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="L18"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -806,39 +941,41 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>POOL-070</t>
+          <t>P-TILE</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Install replacement tile</t>
+          <t>Tile repair package</t>
         </is>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E19" s="1">
         <v>46064</v>
       </c>
       <c r="F19" s="1">
-        <v>46066</v>
+        <v>46070</v>
       </c>
       <c r="G19" s="1">
-        <v>46065</v>
+        <v>46063</v>
       </c>
       <c r="H19" s="1">
-        <v>46067</v>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>17FS</t>
-        </is>
-      </c>
+        <v>46071</v>
+      </c>
+      <c r="I19"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="L19"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -848,39 +985,45 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>POOL-080</t>
+          <t>P-005</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Deck coating touch-up</t>
+          <t>Remove damaged tile</t>
         </is>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E20" s="1">
-        <v>46067</v>
+        <v>46064</v>
       </c>
       <c r="F20" s="1">
-        <v>46069</v>
+        <v>46065</v>
       </c>
       <c r="G20" s="1">
-        <v>46066</v>
+        <v>46063</v>
       </c>
       <c r="H20" s="1">
-        <v>46070</v>
+        <v>46064</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>18FS</t>
+          <t>17FS</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="L20"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -890,25 +1033,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>POOL-090</t>
+          <t>P-006</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Final inspection</t>
+          <t>Install replacement tile</t>
         </is>
       </c>
       <c r="D21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" s="1">
-        <v>46070</v>
+        <v>46066</v>
       </c>
       <c r="F21" s="1">
         <v>46070</v>
       </c>
       <c r="G21" s="1">
-        <v>46071</v>
+        <v>46069</v>
       </c>
       <c r="H21" s="1">
         <v>46071</v>
@@ -920,10 +1063,213 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="L21"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sample Pool Repairs</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>P-007</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Optional owner walkthrough</t>
+        </is>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22" s="1">
+        <v>46071</v>
+      </c>
+      <c r="F22" s="1">
+        <v>46071</v>
+      </c>
+      <c r="G22" s="1">
+        <v>46072</v>
+      </c>
+      <c r="H22" s="1">
+        <v>46072</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>20FS</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sample Pool Repairs</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>P-008</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Deck coating touch-up</t>
+        </is>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23" s="1">
+        <v>46071</v>
+      </c>
+      <c r="F23" s="1">
+        <v>46073</v>
+      </c>
+      <c r="G23" s="1">
+        <v>46070</v>
+      </c>
+      <c r="H23" s="1">
+        <v>46072</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>17SS</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="L23"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sample Pool Repairs</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>P-SPEND-01</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Update pool budget tracker</t>
+        </is>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24" s="1">
+        <v>46072</v>
+      </c>
+      <c r="F24" s="1">
+        <v>46072</v>
+      </c>
+      <c r="G24" s="1">
+        <v>46073</v>
+      </c>
+      <c r="H24" s="1">
+        <v>46073</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>20FS</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="L24"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sample Pool Repairs</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>P-009</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Final pool inspection milestone</t>
+        </is>
+      </c>
+      <c r="D25">
+        <v>2</v>
+      </c>
+      <c r="E25" s="1">
+        <v>46076</v>
+      </c>
+      <c r="F25" s="1">
+        <v>46076</v>
+      </c>
+      <c r="G25" s="1">
+        <v>46077</v>
+      </c>
+      <c r="H25" s="1">
+        <v>46077</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>20FS,22FS</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="L25"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L25"/>
 </worksheet>
 </file>
</xml_diff>